<commit_message>
feat: them campus detection, format Excel moi, them cac script tien ich
- Them CAMPUS_MAP + extract_campus() nhan dien Ha Noi/TP.HCM/Can Tho/Da Nang/Quy Nhon
- Them COL_WIDTHS va COLS dinh nghia format bang Excel chuan
- Them cap_nhat_tom_tat.py, check_html.py, lich_su.py, sync_xlsx.py
- Them Lay-lich-su.bat chay nhanh tren Windows
- Them output folder Trang web FPT/ voi data mau

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Trang web FPT/fpt_news_20260514.xlsx
+++ b/Trang web FPT/fpt_news_20260514.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Tong quan nguon" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Tat ca bai viet" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="20 bai moi nhat" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tong quan nguon" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tat ca bai viet" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="20 bai moi nhat" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -471,7 +471,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>14/05/2026 13:51</t>
+          <t>14/05/2026 13:42</t>
         </is>
       </c>
     </row>
@@ -561,22 +561,22 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>14/05/2026 13:51</t>
+          <t>14/05/2026 13:42</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Nam sinh vùng cao Hà Giang giành học bổng Tiến sĩ toàn phần hơn 7,5 tỷ đồng tại Mỹ</t>
+          <t>Nam sinh vùng cao giành học bổng tiến sĩ toàn phần hơn 7,5 tỷ đồng tại Mỹ</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>VTV.vn &amp;#8211; Từ một cậu học trò rụt rè ở vùng cao, Nguyễn Hồng Anh vừa xuất sắc giành học bổng Tiến sĩ toàn phần trị giá hơn 7,5 tỷ đồng tại Texas Tech University (Mỹ). Nguyễn Hồng Anh là một trong số ít sinh viên Việt Nam nhận được Distinguished Graduate Student Assistantship (DGSA) [&amp;#8230;]</t>
+          <t>Từ học sinh vùng cao rụt rè, Nguyễn Hồng Anh theo đuổi ngành Trí tuệ nhân tạo và xuất sắc giành học bổng tiến sĩ toàn phần Mỹ trị giá 300.000 USD. Sinh ra và lớn lên tại tỉnh vùng cao Tuyên Quang (Hà Giang cũ), nơi điều kiện tiếp cận tri thức và công [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/nam-sinh-vung-cao-ha-giang-gianh-hoc-bong-tien-si-toan-phan-hon-75-ty-dong-tai-my/</t>
+          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/nam-sinh-vung-cao-gianh-hoc-bong-tien-si-toan-phan-hon-75-ty-dong-tai-my/</t>
         </is>
       </c>
     </row>
@@ -588,22 +588,22 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>14/05/2026 13:47</t>
+          <t>13/05/2026 17:01</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Cựu sinh viên FPTU hỗ trợ doanh nghiệp ôtô Mỹ chuyển đổi AI</t>
+          <t>Trường Đại học FPT tổ chức hội thảo phụ huynh quy tụ chuyên gia đa lĩnh vực, cùng giải bài toán nghề nghiệp trong kỷ nguyên AI</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Kỹ sư công nghệ, chuyên gia AI tập đoàn FPT dẫn dắt chuyển đổi AI cho doanh nghiệp lớn ngành công nghiệp ôtô Mỹ, nhằm cải thiện hiệu suất và chất lượng hệ thống. Vũ Minh Phong &amp;#8211; cựu sinh viên K4 chuyên ngành Kỹ thuật phần mềm Trường Đại học FPT &amp;#8211; đã có [&amp;#8230;]</t>
+          <t>Khi trí tuệ nhân tạo (AI) đang thay đổi cách con người học tập, làm việc và phát triển sự nghiệp, nhiều phụ huynh và học sinh đứng trước không ít băn khoăn: Ngành nghề nào sẽ phát triển mạnh trong tương lai? Những công việc nào có nguy cơ bị AI thay thế? Học [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/alumni/cuu-sinh-vien-fptu-ho-tro-doanh-nghiep-oto-my-chuyen-doi-ai/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/truong-dai-hoc-fpt-to-chuc-hoi-thao-phu-huynh-quy-tu-chuyen-gia-da-linh-vuc-cung-giai-bai-toan-nghe-nghiep-trong-ky-nguyen-ai/</t>
         </is>
       </c>
     </row>
@@ -615,49 +615,49 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>14/05/2026 13:42</t>
+          <t>13/05/2026 17:00</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Nam sinh vùng cao giành học bổng tiến sĩ toàn phần hơn 7,5 tỷ đồng tại Mỹ</t>
+          <t>Cựu sinh viên FPTU giành học bổng Tiến sĩ hơn 7,5 tỷ đồng tại Mỹ</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>Từ học sinh vùng cao rụt rè, Nguyễn Hồng Anh theo đuổi ngành Trí tuệ nhân tạo và xuất sắc giành học bổng tiến sĩ toàn phần Mỹ trị giá 300.000 USD. Sinh ra và lớn lên tại tỉnh vùng cao Tuyên Quang (Hà Giang cũ), nơi điều kiện tiếp cận tri thức và công [&amp;#8230;]</t>
+          <t>Nguyễn Hồng Anh, sinh năm 2002, cựu sinh viên trường Đại học FPT (FPTU), nhận học bổng Tiến sĩ toàn phần trị giá khoảng 300.000 USD tại Đại học công nghệ Texas (Mỹ). Từ một học sinh vùng cao Hà Giang từng tự ti trước đám đông, Hồng Anh trở thành một trong những sinh [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/nam-sinh-vung-cao-gianh-hoc-bong-tien-si-toan-phan-hon-75-ty-dong-tai-my/</t>
+          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/cuu-sinh-vien-fptu-gianh-hoc-bong-tien-si-hon-75-ty-dong-tai-my/</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Tin tuc</t>
+          <t>Su kien</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>13/05/2026 17:01</t>
+          <t>13/05/2026 16:35</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Trường Đại học FPT tổ chức hội thảo phụ huynh quy tụ chuyên gia đa lĩnh vực, cùng giải bài toán nghề nghiệp trong kỷ nguyên AI</t>
+          <t>FPTU FUTURE READY TALK 2026: Đồng hành cùng phụ huynh và học sinh trước kỳ tuyển sinh đại học</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Khi trí tuệ nhân tạo (AI) đang thay đổi cách con người học tập, làm việc và phát triển sự nghiệp, nhiều phụ huynh và học sinh đứng trước không ít băn khoăn: Ngành nghề nào sẽ phát triển mạnh trong tương lai? Những công việc nào có nguy cơ bị AI thay thế? Học [&amp;#8230;]</t>
+          <t>Trong bối cảnh AI và công nghệ đang tạo ra nhiều thay đổi mạnh mẽ đối với thị trường lao động và xu hướng nghề nghiệp, việc lựa chọn ngành học và môi trường đào tạo phù hợp trở thành mối quan tâm lớn của nhiều phụ huynh và học sinh lớp 12 trước kỳ [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-tuc/truong-dai-hoc-fpt-to-chuc-hoi-thao-phu-huynh-quy-tu-chuyen-gia-da-linh-vuc-cung-giai-bai-toan-nghe-nghiep-trong-ky-nguyen-ai/</t>
+          <t>https://daihoc.fpt.edu.vn/event/fptu-future-ready-talk-2026-dong-hanh-cung-phu-huynh-va-hoc-sinh-truoc-ky-tuyen-sinh-dai-hoc/</t>
         </is>
       </c>
     </row>
@@ -669,49 +669,49 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>13/05/2026 17:00</t>
+          <t>13/05/2026 14:34</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Cựu sinh viên FPTU giành học bổng Tiến sĩ hơn 7,5 tỷ đồng tại Mỹ</t>
+          <t>Đồ án khởi nghiệp của sinh viên FPTU đạt doanh thu gần 1 tỷ đồng sau 1 năm</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Nguyễn Hồng Anh, sinh năm 2002, cựu sinh viên trường Đại học FPT (FPTU), nhận học bổng Tiến sĩ toàn phần trị giá khoảng 300.000 USD tại Đại học công nghệ Texas (Mỹ). Từ một học sinh vùng cao Hà Giang từng tự ti trước đám đông, Hồng Anh trở thành một trong những sinh [&amp;#8230;]</t>
+          <t>Từ một dự án trong học phần khởi nghiệp tại FPTU, FTES đã phát triển thành nền tảng AI Learning thu hút hơn 4.000 học viên và đạt doanh thu gần 1 tỷ đồng chỉ sau hơn một năm vận hành. Được triển khai từ tháng 3/2025 đến nay, FTES (First Technology Education Solution) &amp;#8211; [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/cuu-sinh-vien-fptu-gianh-hoc-bong-tien-si-hon-75-ty-dong-tai-my/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/do-an-khoi-nghiep-cua-sinh-vien-fptu-dat-doanh-thu-gan-1-ty-dong-sau-1-nam/</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>Su kien</t>
+          <t>Tin tuc</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>13/05/2026 16:35</t>
+          <t>13/05/2026 13:24</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>FPTU FUTURE READY TALK 2026: Đồng hành cùng phụ huynh và học sinh trước kỳ tuyển sinh đại học</t>
+          <t>Cựu sinh viên Trường Đại học FPT kể chuyện làm truyền thông tại DHG Pharma</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Trong bối cảnh AI và công nghệ đang tạo ra nhiều thay đổi mạnh mẽ đối với thị trường lao động và xu hướng nghề nghiệp, việc lựa chọn ngành học và môi trường đào tạo phù hợp trở thành mối quan tâm lớn của nhiều phụ huynh và học sinh lớp 12 trước kỳ [&amp;#8230;]</t>
+          <t>Cựu sinh viên Trường Đại học FPT &amp;#8211; Phan Khương Hoan chia sẻ hành trình làm truyền thông tại DHG Pharma với nhiều hoạt động ý nghĩa vì cộng đồng. Không phải ánh đèn sân khấu hay những chiến dịch truyền thông hào nhoáng, hành trình làm nghề của Phan Khương Hoan lại bắt đầu [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/event/fptu-future-ready-talk-2026-dong-hanh-cung-phu-huynh-va-hoc-sinh-truoc-ky-tuyen-sinh-dai-hoc/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/cuu-sinh-vien-truong-dai-hoc-fpt-2/</t>
         </is>
       </c>
     </row>
@@ -723,22 +723,22 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>13/05/2026 14:34</t>
+          <t>13/05/2026 09:59</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Đồ án khởi nghiệp của sinh viên FPTU đạt doanh thu gần 1 tỷ đồng sau 1 năm</t>
+          <t>Nguyện vọng là gì? Cách đăng ký nguyện vọng trực tuyến 2025</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Từ một dự án trong học phần khởi nghiệp tại FPTU, FTES đã phát triển thành nền tảng AI Learning thu hút hơn 4.000 học viên và đạt doanh thu gần 1 tỷ đồng chỉ sau hơn một năm vận hành. Được triển khai từ tháng 3/2025 đến nay, FTES (First Technology Education Solution) &amp;#8211; [&amp;#8230;]</t>
+          <t>Sau khi kỳ thi tốt nghiệp THPT kết thúc, thí sinh bước vào giai đoạn quan trọng nhất: đăng ký nguyện vọng xét tuyển đại học. Đây là thời điểm quyết định lộ trình tương lai của học sinh. Tuy nhiên, việc hiểu rõ bản chất nguyện vọng là gì và thao tác chính xác [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-tuc/do-an-khoi-nghiep-cua-sinh-vien-fptu-dat-doanh-thu-gan-1-ty-dong-sau-1-nam/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/nguyen-vong-la-gi/</t>
         </is>
       </c>
     </row>
@@ -750,22 +750,22 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>13/05/2026 13:24</t>
+          <t>13/05/2026 09:33</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Cựu sinh viên Trường Đại học FPT kể chuyện làm truyền thông tại DHG Pharma</t>
+          <t>Điểm sàn là gì? Điểm sàn với điểm chuẩn khác nhau như thế nào?</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cựu sinh viên Trường Đại học FPT &amp;#8211; Phan Khương Hoan chia sẻ hành trình làm truyền thông tại DHG Pharma với nhiều hoạt động ý nghĩa vì cộng đồng. Không phải ánh đèn sân khấu hay những chiến dịch truyền thông hào nhoáng, hành trình làm nghề của Phan Khương Hoan lại bắt đầu [&amp;#8230;]</t>
+          <t>Thời điểm hiện tại các sĩ tử chắc hẳn đang phải chạy đua nước rút để chuẩn bị cho kì thi tốt nghiệp trung học phổ thông quốc gia sắp tới. Cùng thời điểm này, các trường đại học sẽ công bố điểm sàn đến với các sĩ tử có nguyện vọng xét tuyển vào [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-tuc/cuu-sinh-vien-truong-dai-hoc-fpt-2/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/diem-san-la-gi/</t>
         </is>
       </c>
     </row>
@@ -777,22 +777,22 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>13/05/2026 09:59</t>
+          <t>13/05/2026 09:23</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Nguyện vọng là gì? Cách đăng ký nguyện vọng trực tuyến 2025</t>
+          <t>Đối tượng ưu tiên là gì? Chi tiết về đối tượng ưu tiên tuyển sinh 2026</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Sau khi kỳ thi tốt nghiệp THPT kết thúc, thí sinh bước vào giai đoạn quan trọng nhất: đăng ký nguyện vọng xét tuyển đại học. Đây là thời điểm quyết định lộ trình tương lai của học sinh. Tuy nhiên, việc hiểu rõ bản chất nguyện vọng là gì và thao tác chính xác [&amp;#8230;]</t>
+          <t>Trong lộ trình xét tuyển đại học, việc nắm rõ đối tượng ưu tiên là gì đóng vai trò cực kỳ quan trọng, giúp học sinh không bỏ lỡ những quyền lợi chính đáng về điểm số. Đây là yếu tố có thể thay đổi cục diện, giúp học sinh gia tăng cơ hội trúng [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/nguyen-vong-la-gi/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/doi-tuong-uu-tien-la-gi/</t>
         </is>
       </c>
     </row>
@@ -804,22 +804,22 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>13/05/2026 09:33</t>
+          <t>13/05/2026 09:12</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>Điểm sàn là gì? Điểm sàn với điểm chuẩn khác nhau như thế nào?</t>
+          <t>Thứ tự nguyện vọng là gì? Những lưu ý khi đăng ký nguyện vọng</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Thời điểm hiện tại các sĩ tử chắc hẳn đang phải chạy đua nước rút để chuẩn bị cho kì thi tốt nghiệp trung học phổ thông quốc gia sắp tới. Cùng thời điểm này, các trường đại học sẽ công bố điểm sàn đến với các sĩ tử có nguyện vọng xét tuyển vào [&amp;#8230;]</t>
+          <t>Thứ tự nguyện vọng là gì? Đây là câu hỏi mà hầu hết học sinh lớp 12 đều quan tâm khi bước vào giai đoạn nước rút của kỳ thi tốt nghiệp THPT và xét tuyển đại học. Việc hiểu đúng bản chất và quy tắc sắp xếp nguyện vọng không chỉ giúp các em [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/diem-san-la-gi/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/thu-tu-nguyen-vong-la-gi/</t>
         </is>
       </c>
     </row>
@@ -831,22 +831,22 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>13/05/2026 09:23</t>
+          <t>12/05/2026 11:29</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>Đối tượng ưu tiên là gì? Chi tiết về đối tượng ưu tiên tuyển sinh 2026</t>
+          <t>Trường ĐH FPT tổ chức Hội nghị quốc tế EAI FISAT 2026</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Trong lộ trình xét tuyển đại học, việc nắm rõ đối tượng ưu tiên là gì đóng vai trò cực kỳ quan trọng, giúp học sinh không bỏ lỡ những quyền lợi chính đáng về điểm số. Đây là yếu tố có thể thay đổi cục diện, giúp học sinh gia tăng cơ hội trúng [&amp;#8230;]</t>
+          <t>Trường ĐH FPT sẽ tổ chức Hội nghị khoa học quốc tế EAI FISAT tại phân hiệu TP. Hồ Chí Minh từ ngày 25-27/11. Sự kiện dự kiến quy tụ hơn 150 chuyên gia trong và ngoài nước, các sinh viên, nghiên cứu sinh về hệ thống thông minh và các kỹ thuật nâng cao [&amp;#8230;]</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/doi-tuong-uu-tien-la-gi/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/truong-dh-fpt-to-chuc-hoi-nghi-quoc-te-eai-fisat-2026/</t>
         </is>
       </c>
     </row>
@@ -1420,22 +1420,22 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026 13:51</t>
+          <t>14/05/2026 13:42</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>Nam sinh vùng cao Hà Giang giành học bổng Tiến sĩ toàn phần hơn 7,5 tỷ đồng tại Mỹ</t>
+          <t>Nam sinh vùng cao giành học bổng tiến sĩ toàn phần hơn 7,5 tỷ đồng tại Mỹ</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>VTV.vn &amp;#8211; Từ một cậu học trò rụt rè ở vùng cao, Nguyễn Hồng Anh vừa xuất sắc giành học bổng Tiến sĩ toàn phần trị giá hơn 7,5 tỷ đồng tại Texas Tech University (Mỹ). Nguyễn Hồng Anh là một trong số ít sinh viên Việt Nam nhận được Distinguished Graduate Student Assistantship (DGSA) [&amp;#8230;]</t>
+          <t>Từ học sinh vùng cao rụt rè, Nguyễn Hồng Anh theo đuổi ngành Trí tuệ nhân tạo và xuất sắc giành học bổng tiến sĩ toàn phần Mỹ trị giá 300.000 USD. Sinh ra và lớn lên tại tỉnh vùng cao Tuyên Quang (Hà Giang cũ), nơi điều kiện tiếp cận tri thức và công [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/nam-sinh-vung-cao-ha-giang-gianh-hoc-bong-tien-si-toan-phan-hon-75-ty-dong-tai-my/</t>
+          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/nam-sinh-vung-cao-gianh-hoc-bong-tien-si-toan-phan-hon-75-ty-dong-tai-my/</t>
         </is>
       </c>
     </row>
@@ -1450,22 +1450,22 @@
       </c>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026 13:47</t>
+          <t>13/05/2026 17:01</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>Cựu sinh viên FPTU hỗ trợ doanh nghiệp ôtô Mỹ chuyển đổi AI</t>
+          <t>Trường Đại học FPT tổ chức hội thảo phụ huynh quy tụ chuyên gia đa lĩnh vực, cùng giải bài toán nghề nghiệp trong kỷ nguyên AI</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Kỹ sư công nghệ, chuyên gia AI tập đoàn FPT dẫn dắt chuyển đổi AI cho doanh nghiệp lớn ngành công nghiệp ôtô Mỹ, nhằm cải thiện hiệu suất và chất lượng hệ thống. Vũ Minh Phong &amp;#8211; cựu sinh viên K4 chuyên ngành Kỹ thuật phần mềm Trường Đại học FPT &amp;#8211; đã có [&amp;#8230;]</t>
+          <t>Khi trí tuệ nhân tạo (AI) đang thay đổi cách con người học tập, làm việc và phát triển sự nghiệp, nhiều phụ huynh và học sinh đứng trước không ít băn khoăn: Ngành nghề nào sẽ phát triển mạnh trong tương lai? Những công việc nào có nguy cơ bị AI thay thế? Học [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/alumni/cuu-sinh-vien-fptu-ho-tro-doanh-nghiep-oto-my-chuyen-doi-ai/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/truong-dai-hoc-fpt-to-chuc-hoi-thao-phu-huynh-quy-tu-chuyen-gia-da-linh-vuc-cung-giai-bai-toan-nghe-nghiep-trong-ky-nguyen-ai/</t>
         </is>
       </c>
     </row>
@@ -1480,22 +1480,22 @@
       </c>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>14/05/2026 13:42</t>
+          <t>13/05/2026 17:00</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Nam sinh vùng cao giành học bổng tiến sĩ toàn phần hơn 7,5 tỷ đồng tại Mỹ</t>
+          <t>Cựu sinh viên FPTU giành học bổng Tiến sĩ hơn 7,5 tỷ đồng tại Mỹ</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Từ học sinh vùng cao rụt rè, Nguyễn Hồng Anh theo đuổi ngành Trí tuệ nhân tạo và xuất sắc giành học bổng tiến sĩ toàn phần Mỹ trị giá 300.000 USD. Sinh ra và lớn lên tại tỉnh vùng cao Tuyên Quang (Hà Giang cũ), nơi điều kiện tiếp cận tri thức và công [&amp;#8230;]</t>
+          <t>Nguyễn Hồng Anh, sinh năm 2002, cựu sinh viên trường Đại học FPT (FPTU), nhận học bổng Tiến sĩ toàn phần trị giá khoảng 300.000 USD tại Đại học công nghệ Texas (Mỹ). Từ một học sinh vùng cao Hà Giang từng tự ti trước đám đông, Hồng Anh trở thành một trong những sinh [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/nam-sinh-vung-cao-gianh-hoc-bong-tien-si-toan-phan-hon-75-ty-dong-tai-my/</t>
+          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/cuu-sinh-vien-fptu-gianh-hoc-bong-tien-si-hon-75-ty-dong-tai-my/</t>
         </is>
       </c>
     </row>
@@ -1505,27 +1505,27 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Tin tuc</t>
+          <t>Su kien</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>13/05/2026 17:01</t>
+          <t>13/05/2026 16:35</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Trường Đại học FPT tổ chức hội thảo phụ huynh quy tụ chuyên gia đa lĩnh vực, cùng giải bài toán nghề nghiệp trong kỷ nguyên AI</t>
+          <t>FPTU FUTURE READY TALK 2026: Đồng hành cùng phụ huynh và học sinh trước kỳ tuyển sinh đại học</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Khi trí tuệ nhân tạo (AI) đang thay đổi cách con người học tập, làm việc và phát triển sự nghiệp, nhiều phụ huynh và học sinh đứng trước không ít băn khoăn: Ngành nghề nào sẽ phát triển mạnh trong tương lai? Những công việc nào có nguy cơ bị AI thay thế? Học [&amp;#8230;]</t>
+          <t>Trong bối cảnh AI và công nghệ đang tạo ra nhiều thay đổi mạnh mẽ đối với thị trường lao động và xu hướng nghề nghiệp, việc lựa chọn ngành học và môi trường đào tạo phù hợp trở thành mối quan tâm lớn của nhiều phụ huynh và học sinh lớp 12 trước kỳ [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-tuc/truong-dai-hoc-fpt-to-chuc-hoi-thao-phu-huynh-quy-tu-chuyen-gia-da-linh-vuc-cung-giai-bai-toan-nghe-nghiep-trong-ky-nguyen-ai/</t>
+          <t>https://daihoc.fpt.edu.vn/event/fptu-future-ready-talk-2026-dong-hanh-cung-phu-huynh-va-hoc-sinh-truoc-ky-tuyen-sinh-dai-hoc/</t>
         </is>
       </c>
     </row>
@@ -1540,22 +1540,22 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>13/05/2026 17:00</t>
+          <t>13/05/2026 14:34</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Cựu sinh viên FPTU giành học bổng Tiến sĩ hơn 7,5 tỷ đồng tại Mỹ</t>
+          <t>Đồ án khởi nghiệp của sinh viên FPTU đạt doanh thu gần 1 tỷ đồng sau 1 năm</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Nguyễn Hồng Anh, sinh năm 2002, cựu sinh viên trường Đại học FPT (FPTU), nhận học bổng Tiến sĩ toàn phần trị giá khoảng 300.000 USD tại Đại học công nghệ Texas (Mỹ). Từ một học sinh vùng cao Hà Giang từng tự ti trước đám đông, Hồng Anh trở thành một trong những sinh [&amp;#8230;]</t>
+          <t>Từ một dự án trong học phần khởi nghiệp tại FPTU, FTES đã phát triển thành nền tảng AI Learning thu hút hơn 4.000 học viên và đạt doanh thu gần 1 tỷ đồng chỉ sau hơn một năm vận hành. Được triển khai từ tháng 3/2025 đến nay, FTES (First Technology Education Solution) &amp;#8211; [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/bao-chi-noi-ve-fptu/cuu-sinh-vien-fptu-gianh-hoc-bong-tien-si-hon-75-ty-dong-tai-my/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/do-an-khoi-nghiep-cua-sinh-vien-fptu-dat-doanh-thu-gan-1-ty-dong-sau-1-nam/</t>
         </is>
       </c>
     </row>
@@ -1565,27 +1565,27 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Su kien</t>
+          <t>Tin tuc</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>13/05/2026 16:35</t>
+          <t>13/05/2026 13:24</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>FPTU FUTURE READY TALK 2026: Đồng hành cùng phụ huynh và học sinh trước kỳ tuyển sinh đại học</t>
+          <t>Cựu sinh viên Trường Đại học FPT kể chuyện làm truyền thông tại DHG Pharma</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Trong bối cảnh AI và công nghệ đang tạo ra nhiều thay đổi mạnh mẽ đối với thị trường lao động và xu hướng nghề nghiệp, việc lựa chọn ngành học và môi trường đào tạo phù hợp trở thành mối quan tâm lớn của nhiều phụ huynh và học sinh lớp 12 trước kỳ [&amp;#8230;]</t>
+          <t>Cựu sinh viên Trường Đại học FPT &amp;#8211; Phan Khương Hoan chia sẻ hành trình làm truyền thông tại DHG Pharma với nhiều hoạt động ý nghĩa vì cộng đồng. Không phải ánh đèn sân khấu hay những chiến dịch truyền thông hào nhoáng, hành trình làm nghề của Phan Khương Hoan lại bắt đầu [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/event/fptu-future-ready-talk-2026-dong-hanh-cung-phu-huynh-va-hoc-sinh-truoc-ky-tuyen-sinh-dai-hoc/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/cuu-sinh-vien-truong-dai-hoc-fpt-2/</t>
         </is>
       </c>
     </row>
@@ -1600,22 +1600,22 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>13/05/2026 14:34</t>
+          <t>13/05/2026 09:59</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Đồ án khởi nghiệp của sinh viên FPTU đạt doanh thu gần 1 tỷ đồng sau 1 năm</t>
+          <t>Nguyện vọng là gì? Cách đăng ký nguyện vọng trực tuyến 2025</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Từ một dự án trong học phần khởi nghiệp tại FPTU, FTES đã phát triển thành nền tảng AI Learning thu hút hơn 4.000 học viên và đạt doanh thu gần 1 tỷ đồng chỉ sau hơn một năm vận hành. Được triển khai từ tháng 3/2025 đến nay, FTES (First Technology Education Solution) &amp;#8211; [&amp;#8230;]</t>
+          <t>Sau khi kỳ thi tốt nghiệp THPT kết thúc, thí sinh bước vào giai đoạn quan trọng nhất: đăng ký nguyện vọng xét tuyển đại học. Đây là thời điểm quyết định lộ trình tương lai của học sinh. Tuy nhiên, việc hiểu rõ bản chất nguyện vọng là gì và thao tác chính xác [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-tuc/do-an-khoi-nghiep-cua-sinh-vien-fptu-dat-doanh-thu-gan-1-ty-dong-sau-1-nam/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/nguyen-vong-la-gi/</t>
         </is>
       </c>
     </row>
@@ -1630,22 +1630,22 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>13/05/2026 13:24</t>
+          <t>13/05/2026 09:33</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Cựu sinh viên Trường Đại học FPT kể chuyện làm truyền thông tại DHG Pharma</t>
+          <t>Điểm sàn là gì? Điểm sàn với điểm chuẩn khác nhau như thế nào?</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Cựu sinh viên Trường Đại học FPT &amp;#8211; Phan Khương Hoan chia sẻ hành trình làm truyền thông tại DHG Pharma với nhiều hoạt động ý nghĩa vì cộng đồng. Không phải ánh đèn sân khấu hay những chiến dịch truyền thông hào nhoáng, hành trình làm nghề của Phan Khương Hoan lại bắt đầu [&amp;#8230;]</t>
+          <t>Thời điểm hiện tại các sĩ tử chắc hẳn đang phải chạy đua nước rút để chuẩn bị cho kì thi tốt nghiệp trung học phổ thông quốc gia sắp tới. Cùng thời điểm này, các trường đại học sẽ công bố điểm sàn đến với các sĩ tử có nguyện vọng xét tuyển vào [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-tuc/cuu-sinh-vien-truong-dai-hoc-fpt-2/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/diem-san-la-gi/</t>
         </is>
       </c>
     </row>
@@ -1660,22 +1660,22 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>13/05/2026 09:59</t>
+          <t>13/05/2026 09:23</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>Nguyện vọng là gì? Cách đăng ký nguyện vọng trực tuyến 2025</t>
+          <t>Đối tượng ưu tiên là gì? Chi tiết về đối tượng ưu tiên tuyển sinh 2026</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Sau khi kỳ thi tốt nghiệp THPT kết thúc, thí sinh bước vào giai đoạn quan trọng nhất: đăng ký nguyện vọng xét tuyển đại học. Đây là thời điểm quyết định lộ trình tương lai của học sinh. Tuy nhiên, việc hiểu rõ bản chất nguyện vọng là gì và thao tác chính xác [&amp;#8230;]</t>
+          <t>Trong lộ trình xét tuyển đại học, việc nắm rõ đối tượng ưu tiên là gì đóng vai trò cực kỳ quan trọng, giúp học sinh không bỏ lỡ những quyền lợi chính đáng về điểm số. Đây là yếu tố có thể thay đổi cục diện, giúp học sinh gia tăng cơ hội trúng [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/nguyen-vong-la-gi/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/doi-tuong-uu-tien-la-gi/</t>
         </is>
       </c>
     </row>
@@ -1690,22 +1690,22 @@
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>13/05/2026 09:33</t>
+          <t>13/05/2026 09:12</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Điểm sàn là gì? Điểm sàn với điểm chuẩn khác nhau như thế nào?</t>
+          <t>Thứ tự nguyện vọng là gì? Những lưu ý khi đăng ký nguyện vọng</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Thời điểm hiện tại các sĩ tử chắc hẳn đang phải chạy đua nước rút để chuẩn bị cho kì thi tốt nghiệp trung học phổ thông quốc gia sắp tới. Cùng thời điểm này, các trường đại học sẽ công bố điểm sàn đến với các sĩ tử có nguyện vọng xét tuyển vào [&amp;#8230;]</t>
+          <t>Thứ tự nguyện vọng là gì? Đây là câu hỏi mà hầu hết học sinh lớp 12 đều quan tâm khi bước vào giai đoạn nước rút của kỳ thi tốt nghiệp THPT và xét tuyển đại học. Việc hiểu đúng bản chất và quy tắc sắp xếp nguyện vọng không chỉ giúp các em [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/diem-san-la-gi/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/thu-tu-nguyen-vong-la-gi/</t>
         </is>
       </c>
     </row>
@@ -1720,22 +1720,22 @@
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>13/05/2026 09:23</t>
+          <t>12/05/2026 11:29</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
         <is>
-          <t>Đối tượng ưu tiên là gì? Chi tiết về đối tượng ưu tiên tuyển sinh 2026</t>
+          <t>Trường ĐH FPT tổ chức Hội nghị quốc tế EAI FISAT 2026</t>
         </is>
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Trong lộ trình xét tuyển đại học, việc nắm rõ đối tượng ưu tiên là gì đóng vai trò cực kỳ quan trọng, giúp học sinh không bỏ lỡ những quyền lợi chính đáng về điểm số. Đây là yếu tố có thể thay đổi cục diện, giúp học sinh gia tăng cơ hội trúng [&amp;#8230;]</t>
+          <t>Trường ĐH FPT sẽ tổ chức Hội nghị khoa học quốc tế EAI FISAT tại phân hiệu TP. Hồ Chí Minh từ ngày 25-27/11. Sự kiện dự kiến quy tụ hơn 150 chuyên gia trong và ngoài nước, các sinh viên, nghiên cứu sinh về hệ thống thông minh và các kỹ thuật nâng cao [&amp;#8230;]</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://daihoc.fpt.edu.vn/tin-campus/tin-campus-can-tho/doi-tuong-uu-tien-la-gi/</t>
+          <t>https://daihoc.fpt.edu.vn/tin-tuc/truong-dh-fpt-to-chuc-hoi-nghi-quoc-te-eai-fisat-2026/</t>
         </is>
       </c>
     </row>

</xml_diff>